<commit_message>
Redigitize Geerts 4A and Bloomingdale
</commit_message>
<xml_diff>
--- a/Antibody doses.xlsx
+++ b/Antibody doses.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elber\Documents\git\JSON2SBML\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48F7E3A5-11C9-4B5A-822C-35AE84605770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{077D8877-F3C4-4AAE-9606-F5166219392A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16371" yWindow="0" windowWidth="16629" windowHeight="17880" xr2:uid="{116471A8-54B7-4BBC-8DA4-5C122436A7F8}"/>
+    <workbookView xWindow="-86" yWindow="0" windowWidth="16629" windowHeight="17880" activeTab="2" xr2:uid="{116471A8-54B7-4BBC-8DA4-5C122436A7F8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Gant PK" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="61">
   <si>
     <t>Gantenerumab</t>
   </si>
@@ -199,12 +200,36 @@
   </si>
   <si>
     <t>Ratio ka/Ka</t>
+  </si>
+  <si>
+    <t>half-life</t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>k</t>
+  </si>
+  <si>
+    <t>BBB</t>
+  </si>
+  <si>
+    <t>BCSFB</t>
+  </si>
+  <si>
+    <t>fBBB</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="167" formatCode="0.0000000"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -234,10 +259,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3710,4 +3736,69 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7C2C8C0-52AB-4AD7-99D1-3BE4803BF6EE}">
+  <dimension ref="A2:F4"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="2" max="2" width="9.3828125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.53515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2">
+        <v>21.55</v>
+      </c>
+      <c r="C2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B3">
+        <f>B2*24</f>
+        <v>517.20000000000005</v>
+      </c>
+      <c r="C3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" s="3">
+        <f>LN(2)/B3</f>
+        <v>1.3401917644237148E-3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4">
+        <f>F2/(F2+F3)</f>
+        <v>0.90909090909090917</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>